<commit_message>
Regen: deployment-variant checks, final stats + research_materials, STATUS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research_materials/03_results/breakdown_qtype_dimension.xlsx
+++ b/research_materials/03_results/breakdown_qtype_dimension.xlsx
@@ -459,7 +459,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Built: 2026-10-07 02:47 by src/build_research_materials.py</t>
+          <t>Built: 2026-10-07 02:57 by src/build_research_materials.py</t>
         </is>
       </c>
     </row>
@@ -582,8 +582,12 @@
       <c r="F2" s="3" t="n">
         <v>0.441</v>
       </c>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
+      <c r="G2" s="3" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.039</v>
+      </c>
       <c r="I2" s="3" t="n">
         <v>0.27</v>
       </c>
@@ -615,8 +619,12 @@
       <c r="F3" s="3" t="n">
         <v>0.412</v>
       </c>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
+      <c r="G3" s="3" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.093</v>
+      </c>
       <c r="I3" s="3" t="n">
         <v>0.307</v>
       </c>
@@ -648,8 +656,12 @@
       <c r="F4" s="3" t="n">
         <v>0.423</v>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="G4" s="3" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.051</v>
+      </c>
       <c r="I4" s="3" t="n">
         <v>0.274</v>
       </c>
@@ -681,8 +693,12 @@
       <c r="F5" s="3" t="n">
         <v>0.379</v>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
+      <c r="G5" s="3" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.137</v>
+      </c>
       <c r="I5" s="3" t="n">
         <v>0.3</v>
       </c>
@@ -714,8 +730,12 @@
       <c r="F6" s="3" t="n">
         <v>0.431</v>
       </c>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+      <c r="G6" s="3" t="n">
+        <v>0.301</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.064</v>
+      </c>
       <c r="I6" s="3" t="n">
         <v>0.288</v>
       </c>
@@ -747,8 +767,12 @@
       <c r="F7" s="3" t="n">
         <v>0.474</v>
       </c>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
+      <c r="G7" s="3" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.073</v>
+      </c>
       <c r="I7" s="3" t="n">
         <v>0.312</v>
       </c>
@@ -780,8 +804,12 @@
       <c r="F8" s="3" t="n">
         <v>0.517</v>
       </c>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="G8" s="3" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.032</v>
+      </c>
       <c r="I8" s="3" t="n">
         <v>0.288</v>
       </c>
@@ -813,8 +841,12 @@
       <c r="F9" s="3" t="n">
         <v>0.356</v>
       </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="G9" s="3" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.174</v>
+      </c>
       <c r="I9" s="3" t="n">
         <v>0.336</v>
       </c>
@@ -846,8 +878,12 @@
       <c r="F10" s="3" t="n">
         <v>0.476</v>
       </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="G10" s="3" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.078</v>
+      </c>
       <c r="I10" s="3" t="n">
         <v>0.302</v>
       </c>
@@ -879,8 +915,12 @@
       <c r="F11" s="3" t="n">
         <v>0.493</v>
       </c>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
+      <c r="G11" s="3" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0.063</v>
+      </c>
       <c r="I11" s="3" t="n">
         <v>0.308</v>
       </c>
@@ -912,8 +952,12 @@
       <c r="F12" s="3" t="n">
         <v>0.493</v>
       </c>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
+      <c r="G12" s="3" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0.028</v>
+      </c>
       <c r="I12" s="3" t="n">
         <v>0.283</v>
       </c>
@@ -945,8 +989,12 @@
       <c r="F13" s="3" t="n">
         <v>0.357</v>
       </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
+      <c r="G13" s="3" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0.196</v>
+      </c>
       <c r="I13" s="3" t="n">
         <v>0.339</v>
       </c>
@@ -978,8 +1026,12 @@
       <c r="F14" s="3" t="n">
         <v>0.491</v>
       </c>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
+      <c r="G14" s="3" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I14" s="3" t="n">
         <v>0.362</v>
       </c>
@@ -1011,8 +1063,12 @@
       <c r="F15" s="3" t="n">
         <v>0.538</v>
       </c>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="G15" s="3" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.066</v>
+      </c>
       <c r="I15" s="3" t="n">
         <v>0.433</v>
       </c>
@@ -1044,8 +1100,12 @@
       <c r="F16" s="3" t="n">
         <v>0.552</v>
       </c>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
+      <c r="G16" s="3" t="n">
+        <v>0.374</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.034</v>
+      </c>
       <c r="I16" s="3" t="n">
         <v>0.372</v>
       </c>
@@ -1077,8 +1137,12 @@
       <c r="F17" s="3" t="n">
         <v>0.444</v>
       </c>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
+      <c r="G17" s="3" t="n">
+        <v>0.397</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.136</v>
+      </c>
       <c r="I17" s="3" t="n">
         <v>0.484</v>
       </c>
@@ -6438,8 +6502,12 @@
       <c r="F162" s="3" t="n">
         <v>0.426</v>
       </c>
-      <c r="G162" s="3" t="n"/>
-      <c r="H162" s="3" t="n"/>
+      <c r="G162" s="3" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="H162" s="3" t="n">
+        <v>0.048</v>
+      </c>
       <c r="I162" s="3" t="n">
         <v>0.282</v>
       </c>
@@ -6471,8 +6539,12 @@
       <c r="F163" s="3" t="n">
         <v>0.433</v>
       </c>
-      <c r="G163" s="3" t="n"/>
-      <c r="H163" s="3" t="n"/>
+      <c r="G163" s="3" t="n">
+        <v>0.313</v>
+      </c>
+      <c r="H163" s="3" t="n">
+        <v>0.113</v>
+      </c>
       <c r="I163" s="3" t="n">
         <v>0.325</v>
       </c>
@@ -6504,8 +6576,12 @@
       <c r="F164" s="3" t="n">
         <v>0.471</v>
       </c>
-      <c r="G164" s="3" t="n"/>
-      <c r="H164" s="3" t="n"/>
+      <c r="G164" s="3" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="H164" s="3" t="n">
+        <v>0.063</v>
+      </c>
       <c r="I164" s="3" t="n">
         <v>0.286</v>
       </c>
@@ -6537,8 +6613,12 @@
       <c r="F165" s="3" t="n">
         <v>0.363</v>
       </c>
-      <c r="G165" s="3" t="n"/>
-      <c r="H165" s="3" t="n"/>
+      <c r="G165" s="3" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="H165" s="3" t="n">
+        <v>0.137</v>
+      </c>
       <c r="I165" s="3" t="n">
         <v>0.311</v>
       </c>
@@ -6570,8 +6650,12 @@
       <c r="F166" s="3" t="n">
         <v>0.515</v>
       </c>
-      <c r="G166" s="3" t="n"/>
-      <c r="H166" s="3" t="n"/>
+      <c r="G166" s="3" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="H166" s="3" t="n">
+        <v>0.051</v>
+      </c>
       <c r="I166" s="3" t="n">
         <v>0.313</v>
       </c>
@@ -6603,8 +6687,12 @@
       <c r="F167" s="3" t="n">
         <v>0.474</v>
       </c>
-      <c r="G167" s="3" t="n"/>
-      <c r="H167" s="3" t="n"/>
+      <c r="G167" s="3" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="H167" s="3" t="n">
+        <v>0.07000000000000001</v>
+      </c>
       <c r="I167" s="3" t="n">
         <v>0.341</v>
       </c>
@@ -6636,8 +6724,12 @@
       <c r="F168" s="3" t="n">
         <v>0.523</v>
       </c>
-      <c r="G168" s="3" t="n"/>
-      <c r="H168" s="3" t="n"/>
+      <c r="G168" s="3" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H168" s="3" t="n">
+        <v>0.025</v>
+      </c>
       <c r="I168" s="3" t="n">
         <v>0.311</v>
       </c>
@@ -6669,8 +6761,12 @@
       <c r="F169" s="3" t="n">
         <v>0.386</v>
       </c>
-      <c r="G169" s="3" t="n"/>
-      <c r="H169" s="3" t="n"/>
+      <c r="G169" s="3" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="H169" s="3" t="n">
+        <v>0.158</v>
+      </c>
       <c r="I169" s="3" t="n">
         <v>0.357</v>
       </c>
@@ -6702,8 +6798,12 @@
       <c r="F170" s="3" t="n">
         <v>0.595</v>
       </c>
-      <c r="G170" s="3" t="n"/>
-      <c r="H170" s="3" t="n"/>
+      <c r="G170" s="3" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="H170" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I170" s="3" t="n">
         <v>0.432</v>
       </c>
@@ -6735,8 +6835,12 @@
       <c r="F171" s="3" t="n">
         <v>0.634</v>
       </c>
-      <c r="G171" s="3" t="n"/>
-      <c r="H171" s="3" t="n"/>
+      <c r="G171" s="3" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="H171" s="3" t="n">
+        <v>0.046</v>
+      </c>
       <c r="I171" s="3" t="n">
         <v>0.468</v>
       </c>
@@ -6768,8 +6872,12 @@
       <c r="F172" s="3" t="n">
         <v>0.673</v>
       </c>
-      <c r="G172" s="3" t="n"/>
-      <c r="H172" s="3" t="n"/>
+      <c r="G172" s="3" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="H172" s="3" t="n">
+        <v>0.02</v>
+      </c>
       <c r="I172" s="3" t="n">
         <v>0.41</v>
       </c>
@@ -6801,8 +6909,12 @@
       <c r="F173" s="3" t="n">
         <v>0.621</v>
       </c>
-      <c r="G173" s="3" t="n"/>
-      <c r="H173" s="3" t="n"/>
+      <c r="G173" s="3" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="H173" s="3" t="n">
+        <v>0.165</v>
+      </c>
       <c r="I173" s="3" t="n">
         <v>0.494</v>
       </c>
@@ -6834,8 +6946,12 @@
       <c r="F174" s="3" t="n">
         <v>0.8120000000000001</v>
       </c>
-      <c r="G174" s="3" t="n"/>
-      <c r="H174" s="3" t="n"/>
+      <c r="G174" s="3" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="H174" s="3" t="n">
+        <v>0.026</v>
+      </c>
       <c r="I174" s="3" t="n">
         <v>0.763</v>
       </c>
@@ -6867,8 +6983,12 @@
       <c r="F175" s="3" t="n">
         <v>0.836</v>
       </c>
-      <c r="G175" s="3" t="n"/>
-      <c r="H175" s="3" t="n"/>
+      <c r="G175" s="3" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="H175" s="3" t="n">
+        <v>0.027</v>
+      </c>
       <c r="I175" s="3" t="n">
         <v>0.823</v>
       </c>
@@ -6900,8 +7020,12 @@
       <c r="F176" s="3" t="n">
         <v>0.8169999999999999</v>
       </c>
-      <c r="G176" s="3" t="n"/>
-      <c r="H176" s="3" t="n"/>
+      <c r="G176" s="3" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="H176" s="3" t="n">
+        <v>0.018</v>
+      </c>
       <c r="I176" s="3" t="n">
         <v>0.765</v>
       </c>
@@ -6933,8 +7057,12 @@
       <c r="F177" s="3" t="n">
         <v>0.841</v>
       </c>
-      <c r="G177" s="3" t="n"/>
-      <c r="H177" s="3" t="n"/>
+      <c r="G177" s="3" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="H177" s="3" t="n">
+        <v>0.039</v>
+      </c>
       <c r="I177" s="3" t="n">
         <v>0.831</v>
       </c>
@@ -12886,8 +13014,12 @@
       <c r="F338" s="3" t="n">
         <v>0.431</v>
       </c>
-      <c r="G338" s="3" t="n"/>
-      <c r="H338" s="3" t="n"/>
+      <c r="G338" s="3" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="H338" s="3" t="n">
+        <v>0.06900000000000001</v>
+      </c>
       <c r="I338" s="3" t="n">
         <v>0.297</v>
       </c>
@@ -12919,8 +13051,12 @@
       <c r="F339" s="3" t="n">
         <v>0.451</v>
       </c>
-      <c r="G339" s="3" t="n"/>
-      <c r="H339" s="3" t="n"/>
+      <c r="G339" s="3" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="H339" s="3" t="n">
+        <v>0.098</v>
+      </c>
       <c r="I339" s="3" t="n">
         <v>0.325</v>
       </c>
@@ -12952,8 +13088,12 @@
       <c r="F340" s="3" t="n">
         <v>0.489</v>
       </c>
-      <c r="G340" s="3" t="n"/>
-      <c r="H340" s="3" t="n"/>
+      <c r="G340" s="3" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H340" s="3" t="n">
+        <v>0.057</v>
+      </c>
       <c r="I340" s="3" t="n">
         <v>0.291</v>
       </c>
@@ -12985,8 +13125,12 @@
       <c r="F341" s="3" t="n">
         <v>0.367</v>
       </c>
-      <c r="G341" s="3" t="n"/>
-      <c r="H341" s="3" t="n"/>
+      <c r="G341" s="3" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H341" s="3" t="n">
+        <v>0.181</v>
+      </c>
       <c r="I341" s="3" t="n">
         <v>0.322</v>
       </c>
@@ -13018,8 +13162,12 @@
       <c r="F342" s="3" t="n">
         <v>0.53</v>
       </c>
-      <c r="G342" s="3" t="n"/>
-      <c r="H342" s="3" t="n"/>
+      <c r="G342" s="3" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="H342" s="3" t="n">
+        <v>0.063</v>
+      </c>
       <c r="I342" s="3" t="n">
         <v>0.311</v>
       </c>
@@ -13051,8 +13199,12 @@
       <c r="F343" s="3" t="n">
         <v>0.491</v>
       </c>
-      <c r="G343" s="3" t="n"/>
-      <c r="H343" s="3" t="n"/>
+      <c r="G343" s="3" t="n">
+        <v>0.334</v>
+      </c>
+      <c r="H343" s="3" t="n">
+        <v>0.08500000000000001</v>
+      </c>
       <c r="I343" s="3" t="n">
         <v>0.347</v>
       </c>
@@ -13084,8 +13236,12 @@
       <c r="F344" s="3" t="n">
         <v>0.527</v>
       </c>
-      <c r="G344" s="3" t="n"/>
-      <c r="H344" s="3" t="n"/>
+      <c r="G344" s="3" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="H344" s="3" t="n">
+        <v>0.026</v>
+      </c>
       <c r="I344" s="3" t="n">
         <v>0.303</v>
       </c>
@@ -13117,8 +13273,12 @@
       <c r="F345" s="3" t="n">
         <v>0.405</v>
       </c>
-      <c r="G345" s="3" t="n"/>
-      <c r="H345" s="3" t="n"/>
+      <c r="G345" s="3" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="H345" s="3" t="n">
+        <v>0.145</v>
+      </c>
       <c r="I345" s="3" t="n">
         <v>0.367</v>
       </c>
@@ -13150,8 +13310,12 @@
       <c r="F346" s="3" t="n">
         <v>0.619</v>
       </c>
-      <c r="G346" s="3" t="n"/>
-      <c r="H346" s="3" t="n"/>
+      <c r="G346" s="3" t="n">
+        <v>0.405</v>
+      </c>
+      <c r="H346" s="3" t="n">
+        <v>0.031</v>
+      </c>
       <c r="I346" s="3" t="n">
         <v>0.37</v>
       </c>
@@ -13183,8 +13347,12 @@
       <c r="F347" s="3" t="n">
         <v>0.613</v>
       </c>
-      <c r="G347" s="3" t="n"/>
-      <c r="H347" s="3" t="n"/>
+      <c r="G347" s="3" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="H347" s="3" t="n">
+        <v>0.05</v>
+      </c>
       <c r="I347" s="3" t="n">
         <v>0.383</v>
       </c>
@@ -13216,8 +13384,12 @@
       <c r="F348" s="3" t="n">
         <v>0.62</v>
       </c>
-      <c r="G348" s="3" t="n"/>
-      <c r="H348" s="3" t="n"/>
+      <c r="G348" s="3" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H348" s="3" t="n">
+        <v>0.022</v>
+      </c>
       <c r="I348" s="3" t="n">
         <v>0.308</v>
       </c>
@@ -13249,8 +13421,12 @@
       <c r="F349" s="3" t="n">
         <v>0.486</v>
       </c>
-      <c r="G349" s="3" t="n"/>
-      <c r="H349" s="3" t="n"/>
+      <c r="G349" s="3" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="H349" s="3" t="n">
+        <v>0.171</v>
+      </c>
       <c r="I349" s="3" t="n">
         <v>0.388</v>
       </c>
@@ -13282,8 +13458,12 @@
       <c r="F350" s="3" t="n">
         <v>0.67</v>
       </c>
-      <c r="G350" s="3" t="n"/>
-      <c r="H350" s="3" t="n"/>
+      <c r="G350" s="3" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="H350" s="3" t="n">
+        <v>0.024</v>
+      </c>
       <c r="I350" s="3" t="n">
         <v>0.554</v>
       </c>
@@ -13315,8 +13495,12 @@
       <c r="F351" s="3" t="n">
         <v>0.698</v>
       </c>
-      <c r="G351" s="3" t="n"/>
-      <c r="H351" s="3" t="n"/>
+      <c r="G351" s="3" t="n">
+        <v>0.537</v>
+      </c>
+      <c r="H351" s="3" t="n">
+        <v>0.026</v>
+      </c>
       <c r="I351" s="3" t="n">
         <v>0.6</v>
       </c>
@@ -13348,8 +13532,12 @@
       <c r="F352" s="3" t="n">
         <v>0.668</v>
       </c>
-      <c r="G352" s="3" t="n"/>
-      <c r="H352" s="3" t="n"/>
+      <c r="G352" s="3" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="H352" s="3" t="n">
+        <v>0.027</v>
+      </c>
       <c r="I352" s="3" t="n">
         <v>0.527</v>
       </c>
@@ -13381,8 +13569,12 @@
       <c r="F353" s="3" t="n">
         <v>0.595</v>
       </c>
-      <c r="G353" s="3" t="n"/>
-      <c r="H353" s="3" t="n"/>
+      <c r="G353" s="3" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="H353" s="3" t="n">
+        <v>0.108</v>
+      </c>
       <c r="I353" s="3" t="n">
         <v>0.635</v>
       </c>
@@ -18742,8 +18934,12 @@
       <c r="F498" s="3" t="n">
         <v>0.293</v>
       </c>
-      <c r="G498" s="3" t="n"/>
-      <c r="H498" s="3" t="n"/>
+      <c r="G498" s="3" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="H498" s="3" t="n">
+        <v>0.08699999999999999</v>
+      </c>
       <c r="I498" s="3" t="n">
         <v>0.262</v>
       </c>
@@ -18775,8 +18971,12 @@
       <c r="F499" s="3" t="n">
         <v>0.468</v>
       </c>
-      <c r="G499" s="3" t="n"/>
-      <c r="H499" s="3" t="n"/>
+      <c r="G499" s="3" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="H499" s="3" t="n">
+        <v>0.09</v>
+      </c>
       <c r="I499" s="3" t="n">
         <v>0.289</v>
       </c>
@@ -18808,8 +19008,12 @@
       <c r="F500" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G500" s="3" t="n"/>
-      <c r="H500" s="3" t="n"/>
+      <c r="G500" s="3" t="n">
+        <v>0.492</v>
+      </c>
+      <c r="H500" s="3" t="n">
+        <v>0.117</v>
+      </c>
       <c r="I500" s="3" t="n">
         <v>0.362</v>
       </c>
@@ -18841,8 +19045,12 @@
       <c r="F501" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G501" s="3" t="n"/>
-      <c r="H501" s="3" t="n"/>
+      <c r="G501" s="3" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="H501" s="3" t="n">
+        <v>0.08799999999999999</v>
+      </c>
       <c r="I501" s="3" t="n">
         <v>0.309</v>
       </c>
@@ -18874,8 +19082,12 @@
       <c r="F502" s="3" t="n">
         <v>0.481</v>
       </c>
-      <c r="G502" s="3" t="n"/>
-      <c r="H502" s="3" t="n"/>
+      <c r="G502" s="3" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H502" s="3" t="n">
+        <v>0.092</v>
+      </c>
       <c r="I502" s="3" t="n">
         <v>0.316</v>
       </c>
@@ -18907,8 +19119,12 @@
       <c r="F503" s="3" t="n">
         <v>0.269</v>
       </c>
-      <c r="G503" s="3" t="n"/>
-      <c r="H503" s="3" t="n"/>
+      <c r="G503" s="3" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="H503" s="3" t="n">
+        <v>0.097</v>
+      </c>
       <c r="I503" s="3" t="n">
         <v>0.254</v>
       </c>
@@ -18940,8 +19156,12 @@
       <c r="F504" s="3" t="n">
         <v>0.339</v>
       </c>
-      <c r="G504" s="3" t="n"/>
-      <c r="H504" s="3" t="n"/>
+      <c r="G504" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H504" s="3" t="n">
+        <v>0.077</v>
+      </c>
       <c r="I504" s="3" t="n">
         <v>0.282</v>
       </c>
@@ -18973,8 +19193,12 @@
       <c r="F505" s="3" t="n">
         <v>0.486</v>
       </c>
-      <c r="G505" s="3" t="n"/>
-      <c r="H505" s="3" t="n"/>
+      <c r="G505" s="3" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="H505" s="3" t="n">
+        <v>0.024</v>
+      </c>
       <c r="I505" s="3" t="n">
         <v>0.309</v>
       </c>
@@ -19006,8 +19230,12 @@
       <c r="F506" s="3" t="n">
         <v>0.385</v>
       </c>
-      <c r="G506" s="3" t="n"/>
-      <c r="H506" s="3" t="n"/>
+      <c r="G506" s="3" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="H506" s="3" t="n">
+        <v>0.06900000000000001</v>
+      </c>
       <c r="I506" s="3" t="n">
         <v>0.295</v>
       </c>
@@ -19039,8 +19267,12 @@
       <c r="F507" s="3" t="n">
         <v>0.333</v>
       </c>
-      <c r="G507" s="3" t="n"/>
-      <c r="H507" s="3" t="n"/>
+      <c r="G507" s="3" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="H507" s="3" t="n">
+        <v>0.08799999999999999</v>
+      </c>
       <c r="I507" s="3" t="n">
         <v>0.263</v>
       </c>
@@ -19072,8 +19304,12 @@
       <c r="F508" s="3" t="n">
         <v>0.365</v>
       </c>
-      <c r="G508" s="3" t="n"/>
-      <c r="H508" s="3" t="n"/>
+      <c r="G508" s="3" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="H508" s="3" t="n">
+        <v>0.08500000000000001</v>
+      </c>
       <c r="I508" s="3" t="n">
         <v>0.272</v>
       </c>
@@ -19105,8 +19341,12 @@
       <c r="F509" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="G509" s="3" t="n"/>
-      <c r="H509" s="3" t="n"/>
+      <c r="G509" s="3" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="H509" s="3" t="n">
+        <v>0.036</v>
+      </c>
       <c r="I509" s="3" t="n">
         <v>0.278</v>
       </c>
@@ -19138,8 +19378,12 @@
       <c r="F510" s="3" t="n">
         <v>0.432</v>
       </c>
-      <c r="G510" s="3" t="n"/>
-      <c r="H510" s="3" t="n"/>
+      <c r="G510" s="3" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="H510" s="3" t="n">
+        <v>0.038</v>
+      </c>
       <c r="I510" s="3" t="n">
         <v>0.273</v>
       </c>
@@ -19171,8 +19415,12 @@
       <c r="F511" s="3" t="n">
         <v>0.322</v>
       </c>
-      <c r="G511" s="3" t="n"/>
-      <c r="H511" s="3" t="n"/>
+      <c r="G511" s="3" t="n">
+        <v>0.201</v>
+      </c>
+      <c r="H511" s="3" t="n">
+        <v>0.149</v>
+      </c>
       <c r="I511" s="3" t="n">
         <v>0.302</v>
       </c>
@@ -19204,8 +19452,12 @@
       <c r="F512" s="3" t="n">
         <v>0.442</v>
       </c>
-      <c r="G512" s="3" t="n"/>
-      <c r="H512" s="3" t="n"/>
+      <c r="G512" s="3" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="H512" s="3" t="n">
+        <v>0.152</v>
+      </c>
       <c r="I512" s="3" t="n">
         <v>0.318</v>
       </c>
@@ -19237,8 +19489,12 @@
       <c r="F513" s="3" t="n">
         <v>0.475</v>
       </c>
-      <c r="G513" s="3" t="n"/>
-      <c r="H513" s="3" t="n"/>
+      <c r="G513" s="3" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="H513" s="3" t="n">
+        <v>0.054</v>
+      </c>
       <c r="I513" s="3" t="n">
         <v>0.292</v>
       </c>
@@ -19270,8 +19526,12 @@
       <c r="F514" s="3" t="n">
         <v>0.453</v>
       </c>
-      <c r="G514" s="3" t="n"/>
-      <c r="H514" s="3" t="n"/>
+      <c r="G514" s="3" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="H514" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I514" s="3" t="n">
         <v>0.314</v>
       </c>
@@ -19303,8 +19563,12 @@
       <c r="F515" s="3" t="n">
         <v>0.404</v>
       </c>
-      <c r="G515" s="3" t="n"/>
-      <c r="H515" s="3" t="n"/>
+      <c r="G515" s="3" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="H515" s="3" t="n">
+        <v>0.073</v>
+      </c>
       <c r="I515" s="3" t="n">
         <v>0.336</v>
       </c>
@@ -19336,8 +19600,12 @@
       <c r="F516" s="3" t="n">
         <v>0.55</v>
       </c>
-      <c r="G516" s="3" t="n"/>
-      <c r="H516" s="3" t="n"/>
+      <c r="G516" s="3" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="H516" s="3" t="n">
+        <v>0.093</v>
+      </c>
       <c r="I516" s="3" t="n">
         <v>0.294</v>
       </c>
@@ -19369,8 +19637,12 @@
       <c r="F517" s="3" t="n">
         <v>0.263</v>
       </c>
-      <c r="G517" s="3" t="n"/>
-      <c r="H517" s="3" t="n"/>
+      <c r="G517" s="3" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="H517" s="3" t="n">
+        <v>0.2</v>
+      </c>
       <c r="I517" s="3" t="n">
         <v>0.302</v>
       </c>
@@ -19402,8 +19674,12 @@
       <c r="F518" s="3" t="n">
         <v>0.344</v>
       </c>
-      <c r="G518" s="3" t="n"/>
-      <c r="H518" s="3" t="n"/>
+      <c r="G518" s="3" t="n">
+        <v>0.302</v>
+      </c>
+      <c r="H518" s="3" t="n">
+        <v>0.108</v>
+      </c>
       <c r="I518" s="3" t="n">
         <v>0.322</v>
       </c>
@@ -19435,8 +19711,12 @@
       <c r="F519" s="3" t="n">
         <v>0.511</v>
       </c>
-      <c r="G519" s="3" t="n"/>
-      <c r="H519" s="3" t="n"/>
+      <c r="G519" s="3" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="H519" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I519" s="3" t="n">
         <v>0.32</v>
       </c>
@@ -19468,8 +19748,12 @@
       <c r="F520" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="G520" s="3" t="n"/>
-      <c r="H520" s="3" t="n"/>
+      <c r="G520" s="3" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H520" s="3" t="n">
+        <v>0.111</v>
+      </c>
       <c r="I520" s="3" t="n">
         <v>0.256</v>
       </c>
@@ -19501,8 +19785,12 @@
       <c r="F521" s="3" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="G521" s="3" t="n"/>
-      <c r="H521" s="3" t="n"/>
+      <c r="G521" s="3" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="H521" s="3" t="n">
+        <v>0.04</v>
+      </c>
       <c r="I521" s="3" t="n">
         <v>0.301</v>
       </c>
@@ -19534,8 +19822,12 @@
       <c r="F522" s="3" t="n">
         <v>0.37</v>
       </c>
-      <c r="G522" s="3" t="n"/>
-      <c r="H522" s="3" t="n"/>
+      <c r="G522" s="3" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="H522" s="3" t="n">
+        <v>0.202</v>
+      </c>
       <c r="I522" s="3" t="n">
         <v>0.322</v>
       </c>
@@ -19567,8 +19859,12 @@
       <c r="F523" s="3" t="n">
         <v>0.517</v>
       </c>
-      <c r="G523" s="3" t="n"/>
-      <c r="H523" s="3" t="n"/>
+      <c r="G523" s="3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H523" s="3" t="n">
+        <v>0.117</v>
+      </c>
       <c r="I523" s="3" t="n">
         <v>0.344</v>
       </c>
@@ -19600,8 +19896,12 @@
       <c r="F524" s="3" t="n">
         <v>0.49</v>
       </c>
-      <c r="G524" s="3" t="n"/>
-      <c r="H524" s="3" t="n"/>
+      <c r="G524" s="3" t="n">
+        <v>0.389</v>
+      </c>
+      <c r="H524" s="3" t="n">
+        <v>0.058</v>
+      </c>
       <c r="I524" s="3" t="n">
         <v>0.322</v>
       </c>
@@ -19633,8 +19933,12 @@
       <c r="F525" s="3" t="n">
         <v>0.333</v>
       </c>
-      <c r="G525" s="3" t="n"/>
-      <c r="H525" s="3" t="n"/>
+      <c r="G525" s="3" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="H525" s="3" t="n">
+        <v>0.097</v>
+      </c>
       <c r="I525" s="3" t="n">
         <v>0.281</v>
       </c>
@@ -19666,8 +19970,12 @@
       <c r="F526" s="3" t="n">
         <v>0.405</v>
       </c>
-      <c r="G526" s="3" t="n"/>
-      <c r="H526" s="3" t="n"/>
+      <c r="G526" s="3" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="H526" s="3" t="n">
+        <v>0.079</v>
+      </c>
       <c r="I526" s="3" t="n">
         <v>0.29</v>
       </c>
@@ -19699,8 +20007,12 @@
       <c r="F527" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G527" s="3" t="n"/>
-      <c r="H527" s="3" t="n"/>
+      <c r="G527" s="3" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="H527" s="3" t="n">
+        <v>0.011</v>
+      </c>
       <c r="I527" s="3" t="n">
         <v>0.303</v>
       </c>
@@ -19732,8 +20044,12 @@
       <c r="F528" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="G528" s="3" t="n"/>
-      <c r="H528" s="3" t="n"/>
+      <c r="G528" s="3" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="H528" s="3" t="n">
+        <v>0.083</v>
+      </c>
       <c r="I528" s="3" t="n">
         <v>0.299</v>
       </c>
@@ -19765,8 +20081,12 @@
       <c r="F529" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="G529" s="3" t="n"/>
-      <c r="H529" s="3" t="n"/>
+      <c r="G529" s="3" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="H529" s="3" t="n">
+        <v>0.133</v>
+      </c>
       <c r="I529" s="3" t="n">
         <v>0.316</v>
       </c>
@@ -19798,8 +20118,12 @@
       <c r="F530" s="3" t="n">
         <v>0.471</v>
       </c>
-      <c r="G530" s="3" t="n"/>
-      <c r="H530" s="3" t="n"/>
+      <c r="G530" s="3" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="H530" s="3" t="n">
+        <v>0.08599999999999999</v>
+      </c>
       <c r="I530" s="3" t="n">
         <v>0.295</v>
       </c>
@@ -19831,8 +20155,12 @@
       <c r="F531" s="3" t="n">
         <v>0.458</v>
       </c>
-      <c r="G531" s="3" t="n"/>
-      <c r="H531" s="3" t="n"/>
+      <c r="G531" s="3" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="H531" s="3" t="n">
+        <v>0.172</v>
+      </c>
       <c r="I531" s="3" t="n">
         <v>0.338</v>
       </c>
@@ -19864,8 +20192,12 @@
       <c r="F532" s="3" t="n">
         <v>0.611</v>
       </c>
-      <c r="G532" s="3" t="n"/>
-      <c r="H532" s="3" t="n"/>
+      <c r="G532" s="3" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="H532" s="3" t="n">
+        <v>0.045</v>
+      </c>
       <c r="I532" s="3" t="n">
         <v>0.402</v>
       </c>
@@ -19897,8 +20229,12 @@
       <c r="F533" s="3" t="n">
         <v>0.392</v>
       </c>
-      <c r="G533" s="3" t="n"/>
-      <c r="H533" s="3" t="n"/>
+      <c r="G533" s="3" t="n">
+        <v>0.394</v>
+      </c>
+      <c r="H533" s="3" t="n">
+        <v>0.125</v>
+      </c>
       <c r="I533" s="3" t="n">
         <v>0.405</v>
       </c>
@@ -19930,8 +20266,12 @@
       <c r="F534" s="3" t="n">
         <v>0.623</v>
       </c>
-      <c r="G534" s="3" t="n"/>
-      <c r="H534" s="3" t="n"/>
+      <c r="G534" s="3" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="H534" s="3" t="n">
+        <v>0.032</v>
+      </c>
       <c r="I534" s="3" t="n">
         <v>0.522</v>
       </c>
@@ -19963,8 +20303,12 @@
       <c r="F535" s="3" t="n">
         <v>0.517</v>
       </c>
-      <c r="G535" s="3" t="n"/>
-      <c r="H535" s="3" t="n"/>
+      <c r="G535" s="3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="H535" s="3" t="n">
+        <v>0.043</v>
+      </c>
       <c r="I535" s="3" t="n">
         <v>0.418</v>
       </c>
@@ -19996,8 +20340,12 @@
       <c r="F536" s="3" t="n">
         <v>0.442</v>
       </c>
-      <c r="G536" s="3" t="n"/>
-      <c r="H536" s="3" t="n"/>
+      <c r="G536" s="3" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="H536" s="3" t="n">
+        <v>0.06</v>
+      </c>
       <c r="I536" s="3" t="n">
         <v>0.392</v>
       </c>
@@ -20029,8 +20377,12 @@
       <c r="F537" s="3" t="n">
         <v>0.486</v>
       </c>
-      <c r="G537" s="3" t="n"/>
-      <c r="H537" s="3" t="n"/>
+      <c r="G537" s="3" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="H537" s="3" t="n">
+        <v>0.106</v>
+      </c>
       <c r="I537" s="3" t="n">
         <v>0.404</v>
       </c>
@@ -20062,8 +20414,12 @@
       <c r="F538" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G538" s="3" t="n"/>
-      <c r="H538" s="3" t="n"/>
+      <c r="G538" s="3" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="H538" s="3" t="n">
+        <v>0.046</v>
+      </c>
       <c r="I538" s="3" t="n">
         <v>0.436</v>
       </c>
@@ -20095,8 +20451,12 @@
       <c r="F539" s="3" t="n">
         <v>0.406</v>
       </c>
-      <c r="G539" s="3" t="n"/>
-      <c r="H539" s="3" t="n"/>
+      <c r="G539" s="3" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="H539" s="3" t="n">
+        <v>0.054</v>
+      </c>
       <c r="I539" s="3" t="n">
         <v>0.388</v>
       </c>
@@ -20128,8 +20488,12 @@
       <c r="F540" s="3" t="n">
         <v>0.522</v>
       </c>
-      <c r="G540" s="3" t="n"/>
-      <c r="H540" s="3" t="n"/>
+      <c r="G540" s="3" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="H540" s="3" t="n">
+        <v>0.096</v>
+      </c>
       <c r="I540" s="3" t="n">
         <v>0.446</v>
       </c>
@@ -20161,8 +20525,12 @@
       <c r="F541" s="3" t="n">
         <v>0.478</v>
       </c>
-      <c r="G541" s="3" t="n"/>
-      <c r="H541" s="3" t="n"/>
+      <c r="G541" s="3" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="H541" s="3" t="n">
+        <v>0.082</v>
+      </c>
       <c r="I541" s="3" t="n">
         <v>0.364</v>
       </c>
@@ -34846,8 +35214,12 @@
       <c r="F938" s="3" t="n">
         <v>0.362</v>
       </c>
-      <c r="G938" s="3" t="n"/>
-      <c r="H938" s="3" t="n"/>
+      <c r="G938" s="3" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="H938" s="3" t="n">
+        <v>0.093</v>
+      </c>
       <c r="I938" s="3" t="n">
         <v>0.281</v>
       </c>
@@ -34879,8 +35251,12 @@
       <c r="F939" s="3" t="n">
         <v>0.444</v>
       </c>
-      <c r="G939" s="3" t="n"/>
-      <c r="H939" s="3" t="n"/>
+      <c r="G939" s="3" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="H939" s="3" t="n">
+        <v>0.116</v>
+      </c>
       <c r="I939" s="3" t="n">
         <v>0.303</v>
       </c>
@@ -34912,8 +35288,12 @@
       <c r="F940" s="3" t="n">
         <v>0.333</v>
       </c>
-      <c r="G940" s="3" t="n"/>
-      <c r="H940" s="3" t="n"/>
+      <c r="G940" s="3" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="H940" s="3" t="n">
+        <v>0.083</v>
+      </c>
       <c r="I940" s="3" t="n">
         <v>0.319</v>
       </c>
@@ -34945,8 +35325,12 @@
       <c r="F941" s="3" t="n">
         <v>0.524</v>
       </c>
-      <c r="G941" s="3" t="n"/>
-      <c r="H941" s="3" t="n"/>
+      <c r="G941" s="3" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="H941" s="3" t="n">
+        <v>0.117</v>
+      </c>
       <c r="I941" s="3" t="n">
         <v>0.32</v>
       </c>
@@ -34978,8 +35362,12 @@
       <c r="F942" s="3" t="n">
         <v>0.487</v>
       </c>
-      <c r="G942" s="3" t="n"/>
-      <c r="H942" s="3" t="n"/>
+      <c r="G942" s="3" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="H942" s="3" t="n">
+        <v>0.08500000000000001</v>
+      </c>
       <c r="I942" s="3" t="n">
         <v>0.313</v>
       </c>
@@ -35011,8 +35399,12 @@
       <c r="F943" s="3" t="n">
         <v>0.269</v>
       </c>
-      <c r="G943" s="3" t="n"/>
-      <c r="H943" s="3" t="n"/>
+      <c r="G943" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H943" s="3" t="n">
+        <v>0.058</v>
+      </c>
       <c r="I943" s="3" t="n">
         <v>0.264</v>
       </c>
@@ -35044,8 +35436,12 @@
       <c r="F944" s="3" t="n">
         <v>0.419</v>
       </c>
-      <c r="G944" s="3" t="n"/>
-      <c r="H944" s="3" t="n"/>
+      <c r="G944" s="3" t="n">
+        <v>0.311</v>
+      </c>
+      <c r="H944" s="3" t="n">
+        <v>0.146</v>
+      </c>
       <c r="I944" s="3" t="n">
         <v>0.321</v>
       </c>
@@ -35077,8 +35473,12 @@
       <c r="F945" s="3" t="n">
         <v>0.556</v>
       </c>
-      <c r="G945" s="3" t="n"/>
-      <c r="H945" s="3" t="n"/>
+      <c r="G945" s="3" t="n">
+        <v>0.394</v>
+      </c>
+      <c r="H945" s="3" t="n">
+        <v>0.008999999999999999</v>
+      </c>
       <c r="I945" s="3" t="n">
         <v>0.328</v>
       </c>
@@ -35110,8 +35510,12 @@
       <c r="F946" s="3" t="n">
         <v>0.327</v>
       </c>
-      <c r="G946" s="3" t="n"/>
-      <c r="H946" s="3" t="n"/>
+      <c r="G946" s="3" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="H946" s="3" t="n">
+        <v>0.07199999999999999</v>
+      </c>
       <c r="I946" s="3" t="n">
         <v>0.296</v>
       </c>
@@ -35143,8 +35547,12 @@
       <c r="F947" s="3" t="n">
         <v>0.333</v>
       </c>
-      <c r="G947" s="3" t="n"/>
-      <c r="H947" s="3" t="n"/>
+      <c r="G947" s="3" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="H947" s="3" t="n">
+        <v>0.091</v>
+      </c>
       <c r="I947" s="3" t="n">
         <v>0.312</v>
       </c>
@@ -35176,8 +35584,12 @@
       <c r="F948" s="3" t="n">
         <v>0.374</v>
       </c>
-      <c r="G948" s="3" t="n"/>
-      <c r="H948" s="3" t="n"/>
+      <c r="G948" s="3" t="n">
+        <v>0.232</v>
+      </c>
+      <c r="H948" s="3" t="n">
+        <v>0.1</v>
+      </c>
       <c r="I948" s="3" t="n">
         <v>0.286</v>
       </c>
@@ -35209,8 +35621,12 @@
       <c r="F949" s="3" t="n">
         <v>0.533</v>
       </c>
-      <c r="G949" s="3" t="n"/>
-      <c r="H949" s="3" t="n"/>
+      <c r="G949" s="3" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H949" s="3" t="n">
+        <v>0.056</v>
+      </c>
       <c r="I949" s="3" t="n">
         <v>0.333</v>
       </c>
@@ -35242,8 +35658,12 @@
       <c r="F950" s="3" t="n">
         <v>0.432</v>
       </c>
-      <c r="G950" s="3" t="n"/>
-      <c r="H950" s="3" t="n"/>
+      <c r="G950" s="3" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="H950" s="3" t="n">
+        <v>0.054</v>
+      </c>
       <c r="I950" s="3" t="n">
         <v>0.315</v>
       </c>
@@ -35275,8 +35695,12 @@
       <c r="F951" s="3" t="n">
         <v>0.411</v>
       </c>
-      <c r="G951" s="3" t="n"/>
-      <c r="H951" s="3" t="n"/>
+      <c r="G951" s="3" t="n">
+        <v>0.307</v>
+      </c>
+      <c r="H951" s="3" t="n">
+        <v>0.134</v>
+      </c>
       <c r="I951" s="3" t="n">
         <v>0.326</v>
       </c>
@@ -35308,8 +35732,12 @@
       <c r="F952" s="3" t="n">
         <v>0.417</v>
       </c>
-      <c r="G952" s="3" t="n"/>
-      <c r="H952" s="3" t="n"/>
+      <c r="G952" s="3" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="H952" s="3" t="n">
+        <v>0.124</v>
+      </c>
       <c r="I952" s="3" t="n">
         <v>0.333</v>
       </c>
@@ -35341,8 +35769,12 @@
       <c r="F953" s="3" t="n">
         <v>0.506</v>
       </c>
-      <c r="G953" s="3" t="n"/>
-      <c r="H953" s="3" t="n"/>
+      <c r="G953" s="3" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="H953" s="3" t="n">
+        <v>0.068</v>
+      </c>
       <c r="I953" s="3" t="n">
         <v>0.326</v>
       </c>
@@ -35374,8 +35806,12 @@
       <c r="F954" s="3" t="n">
         <v>0.469</v>
       </c>
-      <c r="G954" s="3" t="n"/>
-      <c r="H954" s="3" t="n"/>
+      <c r="G954" s="3" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="H954" s="3" t="n">
+        <v>0.064</v>
+      </c>
       <c r="I954" s="3" t="n">
         <v>0.341</v>
       </c>
@@ -35407,8 +35843,12 @@
       <c r="F955" s="3" t="n">
         <v>0.538</v>
       </c>
-      <c r="G955" s="3" t="n"/>
-      <c r="H955" s="3" t="n"/>
+      <c r="G955" s="3" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="H955" s="3" t="n">
+        <v>0.065</v>
+      </c>
       <c r="I955" s="3" t="n">
         <v>0.329</v>
       </c>
@@ -35440,8 +35880,12 @@
       <c r="F956" s="3" t="n">
         <v>0.633</v>
       </c>
-      <c r="G956" s="3" t="n"/>
-      <c r="H956" s="3" t="n"/>
+      <c r="G956" s="3" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="H956" s="3" t="n">
+        <v>0.013</v>
+      </c>
       <c r="I956" s="3" t="n">
         <v>0.311</v>
       </c>
@@ -35473,8 +35917,12 @@
       <c r="F957" s="3" t="n">
         <v>0.368</v>
       </c>
-      <c r="G957" s="3" t="n"/>
-      <c r="H957" s="3" t="n"/>
+      <c r="G957" s="3" t="n">
+        <v>0.289</v>
+      </c>
+      <c r="H957" s="3" t="n">
+        <v>0.024</v>
+      </c>
       <c r="I957" s="3" t="n">
         <v>0.29</v>
       </c>
@@ -35506,8 +35954,12 @@
       <c r="F958" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="G958" s="3" t="n"/>
-      <c r="H958" s="3" t="n"/>
+      <c r="G958" s="3" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H958" s="3" t="n">
+        <v>0.103</v>
+      </c>
       <c r="I958" s="3" t="n">
         <v>0.36</v>
       </c>
@@ -35539,8 +35991,12 @@
       <c r="F959" s="3" t="n">
         <v>0.516</v>
       </c>
-      <c r="G959" s="3" t="n"/>
-      <c r="H959" s="3" t="n"/>
+      <c r="G959" s="3" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="H959" s="3" t="n">
+        <v>0.062</v>
+      </c>
       <c r="I959" s="3" t="n">
         <v>0.338</v>
       </c>
@@ -35572,8 +36028,12 @@
       <c r="F960" s="3" t="n">
         <v>0.708</v>
       </c>
-      <c r="G960" s="3" t="n"/>
-      <c r="H960" s="3" t="n"/>
+      <c r="G960" s="3" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="H960" s="3" t="n">
+        <v>0.078</v>
+      </c>
       <c r="I960" s="3" t="n">
         <v>0.44</v>
       </c>
@@ -35605,8 +36065,12 @@
       <c r="F961" s="3" t="n">
         <v>0.74</v>
       </c>
-      <c r="G961" s="3" t="n"/>
-      <c r="H961" s="3" t="n"/>
+      <c r="G961" s="3" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="H961" s="3" t="n">
+        <v>0.036</v>
+      </c>
       <c r="I961" s="3" t="n">
         <v>0.457</v>
       </c>
@@ -35638,8 +36102,12 @@
       <c r="F962" s="3" t="n">
         <v>0.457</v>
       </c>
-      <c r="G962" s="3" t="n"/>
-      <c r="H962" s="3" t="n"/>
+      <c r="G962" s="3" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="H962" s="3" t="n">
+        <v>0.179</v>
+      </c>
       <c r="I962" s="3" t="n">
         <v>0.399</v>
       </c>
@@ -35671,8 +36139,12 @@
       <c r="F963" s="3" t="n">
         <v>0.75</v>
       </c>
-      <c r="G963" s="3" t="n"/>
-      <c r="H963" s="3" t="n"/>
+      <c r="G963" s="3" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="H963" s="3" t="n">
+        <v>0.098</v>
+      </c>
       <c r="I963" s="3" t="n">
         <v>0.536</v>
       </c>
@@ -35704,8 +36176,12 @@
       <c r="F964" s="3" t="n">
         <v>0.656</v>
       </c>
-      <c r="G964" s="3" t="n"/>
-      <c r="H964" s="3" t="n"/>
+      <c r="G964" s="3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="H964" s="3" t="n">
+        <v>0.036</v>
+      </c>
       <c r="I964" s="3" t="n">
         <v>0.447</v>
       </c>
@@ -35737,8 +36213,12 @@
       <c r="F965" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G965" s="3" t="n"/>
-      <c r="H965" s="3" t="n"/>
+      <c r="G965" s="3" t="n">
+        <v>0.352</v>
+      </c>
+      <c r="H965" s="3" t="n">
+        <v>0.078</v>
+      </c>
       <c r="I965" s="3" t="n">
         <v>0.397</v>
       </c>
@@ -35770,8 +36250,12 @@
       <c r="F966" s="3" t="n">
         <v>0.548</v>
       </c>
-      <c r="G966" s="3" t="n"/>
-      <c r="H966" s="3" t="n"/>
+      <c r="G966" s="3" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="H966" s="3" t="n">
+        <v>0.048</v>
+      </c>
       <c r="I966" s="3" t="n">
         <v>0.46</v>
       </c>
@@ -35803,8 +36287,12 @@
       <c r="F967" s="3" t="n">
         <v>0.6840000000000001</v>
       </c>
-      <c r="G967" s="3" t="n"/>
-      <c r="H967" s="3" t="n"/>
+      <c r="G967" s="3" t="n">
+        <v>0.428</v>
+      </c>
+      <c r="H967" s="3" t="n">
+        <v>0.013</v>
+      </c>
       <c r="I967" s="3" t="n">
         <v>0.412</v>
       </c>
@@ -35836,8 +36324,12 @@
       <c r="F968" s="3" t="n">
         <v>0.55</v>
       </c>
-      <c r="G968" s="3" t="n"/>
-      <c r="H968" s="3" t="n"/>
+      <c r="G968" s="3" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="H968" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="I968" s="3" t="n">
         <v>0.471</v>
       </c>
@@ -35869,8 +36361,12 @@
       <c r="F969" s="3" t="n">
         <v>0.62</v>
       </c>
-      <c r="G969" s="3" t="n"/>
-      <c r="H969" s="3" t="n"/>
+      <c r="G969" s="3" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="H969" s="3" t="n">
+        <v>0.127</v>
+      </c>
       <c r="I969" s="3" t="n">
         <v>0.407</v>
       </c>
@@ -35902,8 +36398,12 @@
       <c r="F970" s="3" t="n">
         <v>0.627</v>
       </c>
-      <c r="G970" s="3" t="n"/>
-      <c r="H970" s="3" t="n"/>
+      <c r="G970" s="3" t="n">
+        <v>0.509</v>
+      </c>
+      <c r="H970" s="3" t="n">
+        <v>0.067</v>
+      </c>
       <c r="I970" s="3" t="n">
         <v>0.472</v>
       </c>
@@ -35935,8 +36435,12 @@
       <c r="F971" s="3" t="n">
         <v>0.833</v>
       </c>
-      <c r="G971" s="3" t="n"/>
-      <c r="H971" s="3" t="n"/>
+      <c r="G971" s="3" t="n">
+        <v>0.717</v>
+      </c>
+      <c r="H971" s="3" t="n">
+        <v>0.021</v>
+      </c>
       <c r="I971" s="3" t="n">
         <v>0.8159999999999999</v>
       </c>
@@ -35968,8 +36472,12 @@
       <c r="F972" s="3" t="n">
         <v>0.856</v>
       </c>
-      <c r="G972" s="3" t="n"/>
-      <c r="H972" s="3" t="n"/>
+      <c r="G972" s="3" t="n">
+        <v>0.781</v>
+      </c>
+      <c r="H972" s="3" t="n">
+        <v>0.023</v>
+      </c>
       <c r="I972" s="3" t="n">
         <v>0.772</v>
       </c>
@@ -36001,8 +36509,12 @@
       <c r="F973" s="3" t="n">
         <v>0.784</v>
       </c>
-      <c r="G973" s="3" t="n"/>
-      <c r="H973" s="3" t="n"/>
+      <c r="G973" s="3" t="n">
+        <v>0.694</v>
+      </c>
+      <c r="H973" s="3" t="n">
+        <v>0.042</v>
+      </c>
       <c r="I973" s="3" t="n">
         <v>0.794</v>
       </c>
@@ -36034,8 +36546,12 @@
       <c r="F974" s="3" t="n">
         <v>0.842</v>
       </c>
-      <c r="G974" s="3" t="n"/>
-      <c r="H974" s="3" t="n"/>
+      <c r="G974" s="3" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="H974" s="3" t="n">
+        <v>0.026</v>
+      </c>
       <c r="I974" s="3" t="n">
         <v>0.804</v>
       </c>
@@ -36067,8 +36583,12 @@
       <c r="F975" s="3" t="n">
         <v>0.8139999999999999</v>
       </c>
-      <c r="G975" s="3" t="n"/>
-      <c r="H975" s="3" t="n"/>
+      <c r="G975" s="3" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="H975" s="3" t="n">
+        <v>0.018</v>
+      </c>
       <c r="I975" s="3" t="n">
         <v>0.766</v>
       </c>
@@ -36100,8 +36620,12 @@
       <c r="F976" s="3" t="n">
         <v>0.827</v>
       </c>
-      <c r="G976" s="3" t="n"/>
-      <c r="H976" s="3" t="n"/>
+      <c r="G976" s="3" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H976" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="I976" s="3" t="n">
         <v>0.821</v>
       </c>
@@ -36133,8 +36657,12 @@
       <c r="F977" s="3" t="n">
         <v>0.833</v>
       </c>
-      <c r="G977" s="3" t="n"/>
-      <c r="H977" s="3" t="n"/>
+      <c r="G977" s="3" t="n">
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="H977" s="3" t="n">
+        <v>0.056</v>
+      </c>
       <c r="I977" s="3" t="n">
         <v>0.758</v>
       </c>
@@ -36166,8 +36694,12 @@
       <c r="F978" s="3" t="n">
         <v>0.8090000000000001</v>
       </c>
-      <c r="G978" s="3" t="n"/>
-      <c r="H978" s="3" t="n"/>
+      <c r="G978" s="3" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="H978" s="3" t="n">
+        <v>0.04</v>
+      </c>
       <c r="I978" s="3" t="n">
         <v>0.832</v>
       </c>
@@ -36199,8 +36731,12 @@
       <c r="F979" s="3" t="n">
         <v>0.8120000000000001</v>
       </c>
-      <c r="G979" s="3" t="n"/>
-      <c r="H979" s="3" t="n"/>
+      <c r="G979" s="3" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="H979" s="3" t="n">
+        <v>0.013</v>
+      </c>
       <c r="I979" s="3" t="n">
         <v>0.79</v>
       </c>
@@ -36232,8 +36768,12 @@
       <c r="F980" s="3" t="n">
         <v>0.859</v>
       </c>
-      <c r="G980" s="3" t="n"/>
-      <c r="H980" s="3" t="n"/>
+      <c r="G980" s="3" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="H980" s="3" t="n">
+        <v>0.041</v>
+      </c>
       <c r="I980" s="3" t="n">
         <v>0.837</v>
       </c>
@@ -36265,8 +36805,12 @@
       <c r="F981" s="3" t="n">
         <v>0.823</v>
       </c>
-      <c r="G981" s="3" t="n"/>
-      <c r="H981" s="3" t="n"/>
+      <c r="G981" s="3" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="H981" s="3" t="n">
+        <v>0.023</v>
+      </c>
       <c r="I981" s="3" t="n">
         <v>0.803</v>
       </c>
@@ -52578,8 +53122,12 @@
       <c r="F1422" s="3" t="n">
         <v>0.345</v>
       </c>
-      <c r="G1422" s="3" t="n"/>
-      <c r="H1422" s="3" t="n"/>
+      <c r="G1422" s="3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="H1422" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I1422" s="3" t="n">
         <v>0.288</v>
       </c>
@@ -52611,8 +53159,12 @@
       <c r="F1423" s="3" t="n">
         <v>0.468</v>
       </c>
-      <c r="G1423" s="3" t="n"/>
-      <c r="H1423" s="3" t="n"/>
+      <c r="G1423" s="3" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="H1423" s="3" t="n">
+        <v>0.152</v>
+      </c>
       <c r="I1423" s="3" t="n">
         <v>0.311</v>
       </c>
@@ -52644,8 +53196,12 @@
       <c r="F1424" s="3" t="n">
         <v>0.75</v>
       </c>
-      <c r="G1424" s="3" t="n"/>
-      <c r="H1424" s="3" t="n"/>
+      <c r="G1424" s="3" t="n">
+        <v>0.492</v>
+      </c>
+      <c r="H1424" s="3" t="n">
+        <v>0.083</v>
+      </c>
       <c r="I1424" s="3" t="n">
         <v>0.33</v>
       </c>
@@ -52677,8 +53233,12 @@
       <c r="F1425" s="3" t="n">
         <v>0.508</v>
       </c>
-      <c r="G1425" s="3" t="n"/>
-      <c r="H1425" s="3" t="n"/>
+      <c r="G1425" s="3" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="H1425" s="3" t="n">
+        <v>0.107</v>
+      </c>
       <c r="I1425" s="3" t="n">
         <v>0.329</v>
       </c>
@@ -52710,8 +53270,12 @@
       <c r="F1426" s="3" t="n">
         <v>0.481</v>
       </c>
-      <c r="G1426" s="3" t="n"/>
-      <c r="H1426" s="3" t="n"/>
+      <c r="G1426" s="3" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="H1426" s="3" t="n">
+        <v>0.116</v>
+      </c>
       <c r="I1426" s="3" t="n">
         <v>0.327</v>
       </c>
@@ -52743,8 +53307,12 @@
       <c r="F1427" s="3" t="n">
         <v>0.269</v>
       </c>
-      <c r="G1427" s="3" t="n"/>
-      <c r="H1427" s="3" t="n"/>
+      <c r="G1427" s="3" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="H1427" s="3" t="n">
+        <v>0.09</v>
+      </c>
       <c r="I1427" s="3" t="n">
         <v>0.249</v>
       </c>
@@ -52776,8 +53344,12 @@
       <c r="F1428" s="3" t="n">
         <v>0.419</v>
       </c>
-      <c r="G1428" s="3" t="n"/>
-      <c r="H1428" s="3" t="n"/>
+      <c r="G1428" s="3" t="n">
+        <v>0.289</v>
+      </c>
+      <c r="H1428" s="3" t="n">
+        <v>0.126</v>
+      </c>
       <c r="I1428" s="3" t="n">
         <v>0.313</v>
       </c>
@@ -52809,8 +53381,12 @@
       <c r="F1429" s="3" t="n">
         <v>0.569</v>
       </c>
-      <c r="G1429" s="3" t="n"/>
-      <c r="H1429" s="3" t="n"/>
+      <c r="G1429" s="3" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H1429" s="3" t="n">
+        <v>0.011</v>
+      </c>
       <c r="I1429" s="3" t="n">
         <v>0.32</v>
       </c>
@@ -52842,8 +53418,12 @@
       <c r="F1430" s="3" t="n">
         <v>0.442</v>
       </c>
-      <c r="G1430" s="3" t="n"/>
-      <c r="H1430" s="3" t="n"/>
+      <c r="G1430" s="3" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="H1430" s="3" t="n">
+        <v>0.131</v>
+      </c>
       <c r="I1430" s="3" t="n">
         <v>0.323</v>
       </c>
@@ -52875,8 +53455,12 @@
       <c r="F1431" s="3" t="n">
         <v>0.37</v>
       </c>
-      <c r="G1431" s="3" t="n"/>
-      <c r="H1431" s="3" t="n"/>
+      <c r="G1431" s="3" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="H1431" s="3" t="n">
+        <v>0.089</v>
+      </c>
       <c r="I1431" s="3" t="n">
         <v>0.312</v>
       </c>
@@ -52908,8 +53492,12 @@
       <c r="F1432" s="3" t="n">
         <v>0.37</v>
       </c>
-      <c r="G1432" s="3" t="n"/>
-      <c r="H1432" s="3" t="n"/>
+      <c r="G1432" s="3" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="H1432" s="3" t="n">
+        <v>0.102</v>
+      </c>
       <c r="I1432" s="3" t="n">
         <v>0.296</v>
       </c>
@@ -52941,8 +53529,12 @@
       <c r="F1433" s="3" t="n">
         <v>0.483</v>
       </c>
-      <c r="G1433" s="3" t="n"/>
-      <c r="H1433" s="3" t="n"/>
+      <c r="G1433" s="3" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="H1433" s="3" t="n">
+        <v>0.019</v>
+      </c>
       <c r="I1433" s="3" t="n">
         <v>0.323</v>
       </c>
@@ -52974,8 +53566,12 @@
       <c r="F1434" s="3" t="n">
         <v>0.595</v>
       </c>
-      <c r="G1434" s="3" t="n"/>
-      <c r="H1434" s="3" t="n"/>
+      <c r="G1434" s="3" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="H1434" s="3" t="n">
+        <v>0.094</v>
+      </c>
       <c r="I1434" s="3" t="n">
         <v>0.354</v>
       </c>
@@ -53007,8 +53603,12 @@
       <c r="F1435" s="3" t="n">
         <v>0.367</v>
       </c>
-      <c r="G1435" s="3" t="n"/>
-      <c r="H1435" s="3" t="n"/>
+      <c r="G1435" s="3" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="H1435" s="3" t="n">
+        <v>0.117</v>
+      </c>
       <c r="I1435" s="3" t="n">
         <v>0.32</v>
       </c>
@@ -53040,8 +53640,12 @@
       <c r="F1436" s="3" t="n">
         <v>0.458</v>
       </c>
-      <c r="G1436" s="3" t="n"/>
-      <c r="H1436" s="3" t="n"/>
+      <c r="G1436" s="3" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="H1436" s="3" t="n">
+        <v>0.125</v>
+      </c>
       <c r="I1436" s="3" t="n">
         <v>0.321</v>
       </c>
@@ -53073,8 +53677,12 @@
       <c r="F1437" s="3" t="n">
         <v>0.494</v>
       </c>
-      <c r="G1437" s="3" t="n"/>
-      <c r="H1437" s="3" t="n"/>
+      <c r="G1437" s="3" t="n">
+        <v>0.417</v>
+      </c>
+      <c r="H1437" s="3" t="n">
+        <v>0.055</v>
+      </c>
       <c r="I1437" s="3" t="n">
         <v>0.317</v>
       </c>
@@ -53106,8 +53714,12 @@
       <c r="F1438" s="3" t="n">
         <v>0.422</v>
       </c>
-      <c r="G1438" s="3" t="n"/>
-      <c r="H1438" s="3" t="n"/>
+      <c r="G1438" s="3" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="H1438" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I1438" s="3" t="n">
         <v>0.32</v>
       </c>
@@ -53139,8 +53751,12 @@
       <c r="F1439" s="3" t="n">
         <v>0.538</v>
       </c>
-      <c r="G1439" s="3" t="n"/>
-      <c r="H1439" s="3" t="n"/>
+      <c r="G1439" s="3" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="H1439" s="3" t="n">
+        <v>0.075</v>
+      </c>
       <c r="I1439" s="3" t="n">
         <v>0.358</v>
       </c>
@@ -53172,8 +53788,12 @@
       <c r="F1440" s="3" t="n">
         <v>0.633</v>
       </c>
-      <c r="G1440" s="3" t="n"/>
-      <c r="H1440" s="3" t="n"/>
+      <c r="G1440" s="3" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="H1440" s="3" t="n">
+        <v>0.036</v>
+      </c>
       <c r="I1440" s="3" t="n">
         <v>0.347</v>
       </c>
@@ -53205,8 +53825,12 @@
       <c r="F1441" s="3" t="n">
         <v>0.342</v>
       </c>
-      <c r="G1441" s="3" t="n"/>
-      <c r="H1441" s="3" t="n"/>
+      <c r="G1441" s="3" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="H1441" s="3" t="n">
+        <v>0.124</v>
+      </c>
       <c r="I1441" s="3" t="n">
         <v>0.285</v>
       </c>
@@ -53238,8 +53862,12 @@
       <c r="F1442" s="3" t="n">
         <v>0.438</v>
       </c>
-      <c r="G1442" s="3" t="n"/>
-      <c r="H1442" s="3" t="n"/>
+      <c r="G1442" s="3" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="H1442" s="3" t="n">
+        <v>0.135</v>
+      </c>
       <c r="I1442" s="3" t="n">
         <v>0.356</v>
       </c>
@@ -53271,8 +53899,12 @@
       <c r="F1443" s="3" t="n">
         <v>0.533</v>
       </c>
-      <c r="G1443" s="3" t="n"/>
-      <c r="H1443" s="3" t="n"/>
+      <c r="G1443" s="3" t="n">
+        <v>0.334</v>
+      </c>
+      <c r="H1443" s="3" t="n">
+        <v>0.05</v>
+      </c>
       <c r="I1443" s="3" t="n">
         <v>0.34</v>
       </c>
@@ -53304,8 +53936,12 @@
       <c r="F1444" s="3" t="n">
         <v>0.583</v>
       </c>
-      <c r="G1444" s="3" t="n"/>
-      <c r="H1444" s="3" t="n"/>
+      <c r="G1444" s="3" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H1444" s="3" t="n">
+        <v>0.117</v>
+      </c>
       <c r="I1444" s="3" t="n">
         <v>0.346</v>
       </c>
@@ -53337,8 +53973,12 @@
       <c r="F1445" s="3" t="n">
         <v>0.64</v>
       </c>
-      <c r="G1445" s="3" t="n"/>
-      <c r="H1445" s="3" t="n"/>
+      <c r="G1445" s="3" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="H1445" s="3" t="n">
+        <v>0.04</v>
+      </c>
       <c r="I1445" s="3" t="n">
         <v>0.351</v>
       </c>
@@ -53370,8 +54010,12 @@
       <c r="F1446" s="3" t="n">
         <v>0.609</v>
       </c>
-      <c r="G1446" s="3" t="n"/>
-      <c r="H1446" s="3" t="n"/>
+      <c r="G1446" s="3" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="H1446" s="3" t="n">
+        <v>0.116</v>
+      </c>
       <c r="I1446" s="3" t="n">
         <v>0.404</v>
       </c>
@@ -53403,8 +54047,12 @@
       <c r="F1447" s="3" t="n">
         <v>0.6830000000000001</v>
       </c>
-      <c r="G1447" s="3" t="n"/>
-      <c r="H1447" s="3" t="n"/>
+      <c r="G1447" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H1447" s="3" t="n">
+        <v>0.039</v>
+      </c>
       <c r="I1447" s="3" t="n">
         <v>0.438</v>
       </c>
@@ -53436,8 +54084,12 @@
       <c r="F1448" s="3" t="n">
         <v>0.594</v>
       </c>
-      <c r="G1448" s="3" t="n"/>
-      <c r="H1448" s="3" t="n"/>
+      <c r="G1448" s="3" t="n">
+        <v>0.393</v>
+      </c>
+      <c r="H1448" s="3" t="n">
+        <v>0.036</v>
+      </c>
       <c r="I1448" s="3" t="n">
         <v>0.37</v>
       </c>
@@ -53469,8 +54121,12 @@
       <c r="F1449" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="G1449" s="3" t="n"/>
-      <c r="H1449" s="3" t="n"/>
+      <c r="G1449" s="3" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="H1449" s="3" t="n">
+        <v>0.06900000000000001</v>
+      </c>
       <c r="I1449" s="3" t="n">
         <v>0.267</v>
       </c>
@@ -53502,8 +54158,12 @@
       <c r="F1450" s="3" t="n">
         <v>0.643</v>
       </c>
-      <c r="G1450" s="3" t="n"/>
-      <c r="H1450" s="3" t="n"/>
+      <c r="G1450" s="3" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="H1450" s="3" t="n">
+        <v>0.067</v>
+      </c>
       <c r="I1450" s="3" t="n">
         <v>0.355</v>
       </c>
@@ -53535,8 +54195,12 @@
       <c r="F1451" s="3" t="n">
         <v>0.553</v>
       </c>
-      <c r="G1451" s="3" t="n"/>
-      <c r="H1451" s="3" t="n"/>
+      <c r="G1451" s="3" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="H1451" s="3" t="n">
+        <v>0.059</v>
+      </c>
       <c r="I1451" s="3" t="n">
         <v>0.345</v>
       </c>
@@ -53568,8 +54232,12 @@
       <c r="F1452" s="3" t="n">
         <v>0.45</v>
       </c>
-      <c r="G1452" s="3" t="n"/>
-      <c r="H1452" s="3" t="n"/>
+      <c r="G1452" s="3" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="H1452" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="I1452" s="3" t="n">
         <v>0.308</v>
       </c>
@@ -53601,8 +54269,12 @@
       <c r="F1453" s="3" t="n">
         <v>0.48</v>
       </c>
-      <c r="G1453" s="3" t="n"/>
-      <c r="H1453" s="3" t="n"/>
+      <c r="G1453" s="3" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="H1453" s="3" t="n">
+        <v>0.121</v>
+      </c>
       <c r="I1453" s="3" t="n">
         <v>0.361</v>
       </c>
@@ -53634,8 +54306,12 @@
       <c r="F1454" s="3" t="n">
         <v>0.598</v>
       </c>
-      <c r="G1454" s="3" t="n"/>
-      <c r="H1454" s="3" t="n"/>
+      <c r="G1454" s="3" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="H1454" s="3" t="n">
+        <v>0.089</v>
+      </c>
       <c r="I1454" s="3" t="n">
         <v>0.345</v>
       </c>
@@ -53667,8 +54343,12 @@
       <c r="F1455" s="3" t="n">
         <v>0.667</v>
       </c>
-      <c r="G1455" s="3" t="n"/>
-      <c r="H1455" s="3" t="n"/>
+      <c r="G1455" s="3" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="H1455" s="3" t="n">
+        <v>0.037</v>
+      </c>
       <c r="I1455" s="3" t="n">
         <v>0.608</v>
       </c>
@@ -53700,8 +54380,12 @@
       <c r="F1456" s="3" t="n">
         <v>0.744</v>
       </c>
-      <c r="G1456" s="3" t="n"/>
-      <c r="H1456" s="3" t="n"/>
+      <c r="G1456" s="3" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="H1456" s="3" t="n">
+        <v>0.066</v>
+      </c>
       <c r="I1456" s="3" t="n">
         <v>0.532</v>
       </c>
@@ -53733,8 +54417,12 @@
       <c r="F1457" s="3" t="n">
         <v>0.608</v>
       </c>
-      <c r="G1457" s="3" t="n"/>
-      <c r="H1457" s="3" t="n"/>
+      <c r="G1457" s="3" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="H1457" s="3" t="n">
+        <v>0.052</v>
+      </c>
       <c r="I1457" s="3" t="n">
         <v>0.599</v>
       </c>
@@ -53766,8 +54454,12 @@
       <c r="F1458" s="3" t="n">
         <v>0.763</v>
       </c>
-      <c r="G1458" s="3" t="n"/>
-      <c r="H1458" s="3" t="n"/>
+      <c r="G1458" s="3" t="n">
+        <v>0.704</v>
+      </c>
+      <c r="H1458" s="3" t="n">
+        <v>0.027</v>
+      </c>
       <c r="I1458" s="3" t="n">
         <v>0.671</v>
       </c>
@@ -53799,8 +54491,12 @@
       <c r="F1459" s="3" t="n">
         <v>0.6919999999999999</v>
       </c>
-      <c r="G1459" s="3" t="n"/>
-      <c r="H1459" s="3" t="n"/>
+      <c r="G1459" s="3" t="n">
+        <v>0.507</v>
+      </c>
+      <c r="H1459" s="3" t="n">
+        <v>0.034</v>
+      </c>
       <c r="I1459" s="3" t="n">
         <v>0.594</v>
       </c>
@@ -53832,8 +54528,12 @@
       <c r="F1460" s="3" t="n">
         <v>0.635</v>
       </c>
-      <c r="G1460" s="3" t="n"/>
-      <c r="H1460" s="3" t="n"/>
+      <c r="G1460" s="3" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="H1460" s="3" t="n">
+        <v>0.042</v>
+      </c>
       <c r="I1460" s="3" t="n">
         <v>0.551</v>
       </c>
@@ -53865,8 +54565,12 @@
       <c r="F1461" s="3" t="n">
         <v>0.639</v>
       </c>
-      <c r="G1461" s="3" t="n"/>
-      <c r="H1461" s="3" t="n"/>
+      <c r="G1461" s="3" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="H1461" s="3" t="n">
+        <v>0.06900000000000001</v>
+      </c>
       <c r="I1461" s="3" t="n">
         <v>0.577</v>
       </c>
@@ -53898,8 +54602,12 @@
       <c r="F1462" s="3" t="n">
         <v>0.588</v>
       </c>
-      <c r="G1462" s="3" t="n"/>
-      <c r="H1462" s="3" t="n"/>
+      <c r="G1462" s="3" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="H1462" s="3" t="n">
+        <v>0.021</v>
+      </c>
       <c r="I1462" s="3" t="n">
         <v>0.596</v>
       </c>
@@ -53931,8 +54639,12 @@
       <c r="F1463" s="3" t="n">
         <v>0.5620000000000001</v>
       </c>
-      <c r="G1463" s="3" t="n"/>
-      <c r="H1463" s="3" t="n"/>
+      <c r="G1463" s="3" t="n">
+        <v>0.501</v>
+      </c>
+      <c r="H1463" s="3" t="n">
+        <v>0.021</v>
+      </c>
       <c r="I1463" s="3" t="n">
         <v>0.5590000000000001</v>
       </c>
@@ -53964,8 +54676,12 @@
       <c r="F1464" s="3" t="n">
         <v>0.717</v>
       </c>
-      <c r="G1464" s="3" t="n"/>
-      <c r="H1464" s="3" t="n"/>
+      <c r="G1464" s="3" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="H1464" s="3" t="n">
+        <v>0.095</v>
+      </c>
       <c r="I1464" s="3" t="n">
         <v>0.621</v>
       </c>
@@ -53997,8 +54713,12 @@
       <c r="F1465" s="3" t="n">
         <v>0.5649999999999999</v>
       </c>
-      <c r="G1465" s="3" t="n"/>
-      <c r="H1465" s="3" t="n"/>
+      <c r="G1465" s="3" t="n">
+        <v>0.476</v>
+      </c>
+      <c r="H1465" s="3" t="n">
+        <v>0.044</v>
+      </c>
       <c r="I1465" s="3" t="n">
         <v>0.503</v>
       </c>
@@ -68682,8 +69402,12 @@
       <c r="F1862" s="3" t="n">
         <v>0.382</v>
       </c>
-      <c r="G1862" s="3" t="n"/>
-      <c r="H1862" s="3" t="n"/>
+      <c r="G1862" s="3" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="H1862" s="3" t="n">
+        <v>0.134</v>
+      </c>
       <c r="I1862" s="3" t="n">
         <v>0.3</v>
       </c>
@@ -68715,8 +69439,12 @@
       <c r="F1863" s="3" t="n">
         <v>0.441</v>
       </c>
-      <c r="G1863" s="3" t="n"/>
-      <c r="H1863" s="3" t="n"/>
+      <c r="G1863" s="3" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="H1863" s="3" t="n">
+        <v>0.039</v>
+      </c>
       <c r="I1863" s="3" t="n">
         <v>0.27</v>
       </c>
@@ -68748,8 +69476,12 @@
       <c r="F1864" s="3" t="n">
         <v>0.424</v>
       </c>
-      <c r="G1864" s="3" t="n"/>
-      <c r="H1864" s="3" t="n"/>
+      <c r="G1864" s="3" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="H1864" s="3" t="n">
+        <v>0.06</v>
+      </c>
       <c r="I1864" s="3" t="n">
         <v>0.289</v>
       </c>
@@ -68781,8 +69513,12 @@
       <c r="F1865" s="3" t="n">
         <v>0.377</v>
       </c>
-      <c r="G1865" s="3" t="n"/>
-      <c r="H1865" s="3" t="n"/>
+      <c r="G1865" s="3" t="n">
+        <v>0.299</v>
+      </c>
+      <c r="H1865" s="3" t="n">
+        <v>0.151</v>
+      </c>
       <c r="I1865" s="3" t="n">
         <v>0.327</v>
       </c>
@@ -68814,8 +69550,12 @@
       <c r="F1866" s="3" t="n">
         <v>0.431</v>
       </c>
-      <c r="G1866" s="3" t="n"/>
-      <c r="H1866" s="3" t="n"/>
+      <c r="G1866" s="3" t="n">
+        <v>0.301</v>
+      </c>
+      <c r="H1866" s="3" t="n">
+        <v>0.064</v>
+      </c>
       <c r="I1866" s="3" t="n">
         <v>0.288</v>
       </c>
@@ -68847,8 +69587,12 @@
       <c r="F1867" s="3" t="n">
         <v>0.502</v>
       </c>
-      <c r="G1867" s="3" t="n"/>
-      <c r="H1867" s="3" t="n"/>
+      <c r="G1867" s="3" t="n">
+        <v>0.327</v>
+      </c>
+      <c r="H1867" s="3" t="n">
+        <v>0.05</v>
+      </c>
       <c r="I1867" s="3" t="n">
         <v>0.299</v>
       </c>
@@ -68880,8 +69624,12 @@
       <c r="F1868" s="3" t="n">
         <v>0.392</v>
       </c>
-      <c r="G1868" s="3" t="n"/>
-      <c r="H1868" s="3" t="n"/>
+      <c r="G1868" s="3" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="H1868" s="3" t="n">
+        <v>0.16</v>
+      </c>
       <c r="I1868" s="3" t="n">
         <v>0.334</v>
       </c>
@@ -68913,8 +69661,12 @@
       <c r="F1869" s="3" t="n">
         <v>0.483</v>
       </c>
-      <c r="G1869" s="3" t="n"/>
-      <c r="H1869" s="3" t="n"/>
+      <c r="G1869" s="3" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="H1869" s="3" t="n">
+        <v>0.065</v>
+      </c>
       <c r="I1869" s="3" t="n">
         <v>0.297</v>
       </c>
@@ -68946,8 +69698,12 @@
       <c r="F1870" s="3" t="n">
         <v>0.485</v>
       </c>
-      <c r="G1870" s="3" t="n"/>
-      <c r="H1870" s="3" t="n"/>
+      <c r="G1870" s="3" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="H1870" s="3" t="n">
+        <v>0.055</v>
+      </c>
       <c r="I1870" s="3" t="n">
         <v>0.294</v>
       </c>
@@ -68979,8 +69735,12 @@
       <c r="F1871" s="3" t="n">
         <v>0.484</v>
       </c>
-      <c r="G1871" s="3" t="n"/>
-      <c r="H1871" s="3" t="n"/>
+      <c r="G1871" s="3" t="n">
+        <v>0.442</v>
+      </c>
+      <c r="H1871" s="3" t="n">
+        <v>0.12</v>
+      </c>
       <c r="I1871" s="3" t="n">
         <v>0.485</v>
       </c>
@@ -69012,8 +69772,12 @@
       <c r="F1872" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="G1872" s="3" t="n"/>
-      <c r="H1872" s="3" t="n"/>
+      <c r="G1872" s="3" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="H1872" s="3" t="n">
+        <v>0.049</v>
+      </c>
       <c r="I1872" s="3" t="n">
         <v>0.36</v>
       </c>
@@ -69045,8 +69809,12 @@
       <c r="F1873" s="3" t="n">
         <v>0.528</v>
       </c>
-      <c r="G1873" s="3" t="n"/>
-      <c r="H1873" s="3" t="n"/>
+      <c r="G1873" s="3" t="n">
+        <v>0.369</v>
+      </c>
+      <c r="H1873" s="3" t="n">
+        <v>0.05</v>
+      </c>
       <c r="I1873" s="3" t="n">
         <v>0.389</v>
       </c>
@@ -73074,8 +73842,12 @@
       <c r="F1982" s="3" t="n">
         <v>0.387</v>
       </c>
-      <c r="G1982" s="3" t="n"/>
-      <c r="H1982" s="3" t="n"/>
+      <c r="G1982" s="3" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="H1982" s="3" t="n">
+        <v>0.137</v>
+      </c>
       <c r="I1982" s="3" t="n">
         <v>0.317</v>
       </c>
@@ -73107,8 +73879,12 @@
       <c r="F1983" s="3" t="n">
         <v>0.426</v>
       </c>
-      <c r="G1983" s="3" t="n"/>
-      <c r="H1983" s="3" t="n"/>
+      <c r="G1983" s="3" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="H1983" s="3" t="n">
+        <v>0.048</v>
+      </c>
       <c r="I1983" s="3" t="n">
         <v>0.282</v>
       </c>
@@ -73140,8 +73916,12 @@
       <c r="F1984" s="3" t="n">
         <v>0.453</v>
       </c>
-      <c r="G1984" s="3" t="n"/>
-      <c r="H1984" s="3" t="n"/>
+      <c r="G1984" s="3" t="n">
+        <v>0.321</v>
+      </c>
+      <c r="H1984" s="3" t="n">
+        <v>0.077</v>
+      </c>
       <c r="I1984" s="3" t="n">
         <v>0.3</v>
       </c>
@@ -73173,8 +73953,12 @@
       <c r="F1985" s="3" t="n">
         <v>0.408</v>
       </c>
-      <c r="G1985" s="3" t="n"/>
-      <c r="H1985" s="3" t="n"/>
+      <c r="G1985" s="3" t="n">
+        <v>0.329</v>
+      </c>
+      <c r="H1985" s="3" t="n">
+        <v>0.148</v>
+      </c>
       <c r="I1985" s="3" t="n">
         <v>0.353</v>
       </c>
@@ -73206,8 +73990,12 @@
       <c r="F1986" s="3" t="n">
         <v>0.515</v>
       </c>
-      <c r="G1986" s="3" t="n"/>
-      <c r="H1986" s="3" t="n"/>
+      <c r="G1986" s="3" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="H1986" s="3" t="n">
+        <v>0.051</v>
+      </c>
       <c r="I1986" s="3" t="n">
         <v>0.313</v>
       </c>
@@ -73239,8 +74027,12 @@
       <c r="F1987" s="3" t="n">
         <v>0.502</v>
       </c>
-      <c r="G1987" s="3" t="n"/>
-      <c r="H1987" s="3" t="n"/>
+      <c r="G1987" s="3" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="H1987" s="3" t="n">
+        <v>0.037</v>
+      </c>
       <c r="I1987" s="3" t="n">
         <v>0.323</v>
       </c>
@@ -73272,8 +74064,12 @@
       <c r="F1988" s="3" t="n">
         <v>0.636</v>
       </c>
-      <c r="G1988" s="3" t="n"/>
-      <c r="H1988" s="3" t="n"/>
+      <c r="G1988" s="3" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="H1988" s="3" t="n">
+        <v>0.138</v>
+      </c>
       <c r="I1988" s="3" t="n">
         <v>0.502</v>
       </c>
@@ -73305,8 +74101,12 @@
       <c r="F1989" s="3" t="n">
         <v>0.608</v>
       </c>
-      <c r="G1989" s="3" t="n"/>
-      <c r="H1989" s="3" t="n"/>
+      <c r="G1989" s="3" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="H1989" s="3" t="n">
+        <v>0.042</v>
+      </c>
       <c r="I1989" s="3" t="n">
         <v>0.433</v>
       </c>
@@ -73338,8 +74138,12 @@
       <c r="F1990" s="3" t="n">
         <v>0.641</v>
       </c>
-      <c r="G1990" s="3" t="n"/>
-      <c r="H1990" s="3" t="n"/>
+      <c r="G1990" s="3" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="H1990" s="3" t="n">
+        <v>0.038</v>
+      </c>
       <c r="I1990" s="3" t="n">
         <v>0.425</v>
       </c>
@@ -73371,8 +74175,12 @@
       <c r="F1991" s="3" t="n">
         <v>0.857</v>
       </c>
-      <c r="G1991" s="3" t="n"/>
-      <c r="H1991" s="3" t="n"/>
+      <c r="G1991" s="3" t="n">
+        <v>0.702</v>
+      </c>
+      <c r="H1991" s="3" t="n">
+        <v>0.03</v>
+      </c>
       <c r="I1991" s="3" t="n">
         <v>0.842</v>
       </c>
@@ -73404,8 +74212,12 @@
       <c r="F1992" s="3" t="n">
         <v>0.821</v>
       </c>
-      <c r="G1992" s="3" t="n"/>
-      <c r="H1992" s="3" t="n"/>
+      <c r="G1992" s="3" t="n">
+        <v>0.769</v>
+      </c>
+      <c r="H1992" s="3" t="n">
+        <v>0.022</v>
+      </c>
       <c r="I1992" s="3" t="n">
         <v>0.763</v>
       </c>
@@ -73437,8 +74249,12 @@
       <c r="F1993" s="3" t="n">
         <v>0.8090000000000001</v>
       </c>
-      <c r="G1993" s="3" t="n"/>
-      <c r="H1993" s="3" t="n"/>
+      <c r="G1993" s="3" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="H1993" s="3" t="n">
+        <v>0.028</v>
+      </c>
       <c r="I1993" s="3" t="n">
         <v>0.78</v>
       </c>
@@ -77910,8 +78726,12 @@
       <c r="F2114" s="3" t="n">
         <v>0.387</v>
       </c>
-      <c r="G2114" s="3" t="n"/>
-      <c r="H2114" s="3" t="n"/>
+      <c r="G2114" s="3" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="H2114" s="3" t="n">
+        <v>0.169</v>
+      </c>
       <c r="I2114" s="3" t="n">
         <v>0.32</v>
       </c>
@@ -77943,8 +78763,12 @@
       <c r="F2115" s="3" t="n">
         <v>0.431</v>
       </c>
-      <c r="G2115" s="3" t="n"/>
-      <c r="H2115" s="3" t="n"/>
+      <c r="G2115" s="3" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="H2115" s="3" t="n">
+        <v>0.06900000000000001</v>
+      </c>
       <c r="I2115" s="3" t="n">
         <v>0.297</v>
       </c>
@@ -77976,8 +78800,12 @@
       <c r="F2116" s="3" t="n">
         <v>0.478</v>
       </c>
-      <c r="G2116" s="3" t="n"/>
-      <c r="H2116" s="3" t="n"/>
+      <c r="G2116" s="3" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="H2116" s="3" t="n">
+        <v>0.063</v>
+      </c>
       <c r="I2116" s="3" t="n">
         <v>0.307</v>
       </c>
@@ -78009,8 +78837,12 @@
       <c r="F2117" s="3" t="n">
         <v>0.417</v>
       </c>
-      <c r="G2117" s="3" t="n"/>
-      <c r="H2117" s="3" t="n"/>
+      <c r="G2117" s="3" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="H2117" s="3" t="n">
+        <v>0.136</v>
+      </c>
       <c r="I2117" s="3" t="n">
         <v>0.361</v>
       </c>
@@ -78042,8 +78874,12 @@
       <c r="F2118" s="3" t="n">
         <v>0.53</v>
       </c>
-      <c r="G2118" s="3" t="n"/>
-      <c r="H2118" s="3" t="n"/>
+      <c r="G2118" s="3" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="H2118" s="3" t="n">
+        <v>0.063</v>
+      </c>
       <c r="I2118" s="3" t="n">
         <v>0.311</v>
       </c>
@@ -78075,8 +78911,12 @@
       <c r="F2119" s="3" t="n">
         <v>0.517</v>
       </c>
-      <c r="G2119" s="3" t="n"/>
-      <c r="H2119" s="3" t="n"/>
+      <c r="G2119" s="3" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="H2119" s="3" t="n">
+        <v>0.046</v>
+      </c>
       <c r="I2119" s="3" t="n">
         <v>0.321</v>
       </c>
@@ -78108,8 +78948,12 @@
       <c r="F2120" s="3" t="n">
         <v>0.534</v>
       </c>
-      <c r="G2120" s="3" t="n"/>
-      <c r="H2120" s="3" t="n"/>
+      <c r="G2120" s="3" t="n">
+        <v>0.354</v>
+      </c>
+      <c r="H2120" s="3" t="n">
+        <v>0.144</v>
+      </c>
       <c r="I2120" s="3" t="n">
         <v>0.404</v>
       </c>
@@ -78141,8 +78985,12 @@
       <c r="F2121" s="3" t="n">
         <v>0.625</v>
       </c>
-      <c r="G2121" s="3" t="n"/>
-      <c r="H2121" s="3" t="n"/>
+      <c r="G2121" s="3" t="n">
+        <v>0.403</v>
+      </c>
+      <c r="H2121" s="3" t="n">
+        <v>0.033</v>
+      </c>
       <c r="I2121" s="3" t="n">
         <v>0.369</v>
       </c>
@@ -78174,8 +79022,12 @@
       <c r="F2122" s="3" t="n">
         <v>0.599</v>
       </c>
-      <c r="G2122" s="3" t="n"/>
-      <c r="H2122" s="3" t="n"/>
+      <c r="G2122" s="3" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="H2122" s="3" t="n">
+        <v>0.034</v>
+      </c>
       <c r="I2122" s="3" t="n">
         <v>0.329</v>
       </c>
@@ -78207,8 +79059,12 @@
       <c r="F2123" s="3" t="n">
         <v>0.627</v>
       </c>
-      <c r="G2123" s="3" t="n"/>
-      <c r="H2123" s="3" t="n"/>
+      <c r="G2123" s="3" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="H2123" s="3" t="n">
+        <v>0.092</v>
+      </c>
       <c r="I2123" s="3" t="n">
         <v>0.64</v>
       </c>
@@ -78240,8 +79096,12 @@
       <c r="F2124" s="3" t="n">
         <v>0.679</v>
       </c>
-      <c r="G2124" s="3" t="n"/>
-      <c r="H2124" s="3" t="n"/>
+      <c r="G2124" s="3" t="n">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="H2124" s="3" t="n">
+        <v>0.025</v>
+      </c>
       <c r="I2124" s="3" t="n">
         <v>0.554</v>
       </c>
@@ -78273,8 +79133,12 @@
       <c r="F2125" s="3" t="n">
         <v>0.67</v>
       </c>
-      <c r="G2125" s="3" t="n"/>
-      <c r="H2125" s="3" t="n"/>
+      <c r="G2125" s="3" t="n">
+        <v>0.501</v>
+      </c>
+      <c r="H2125" s="3" t="n">
+        <v>0.025</v>
+      </c>
       <c r="I2125" s="3" t="n">
         <v>0.549</v>
       </c>

</xml_diff>